<commit_message>
Agregando el frontend con React
</commit_message>
<xml_diff>
--- a/assets/Listados/CGS - 3414937 - 2026.xlsx
+++ b/assets/Listados/CGS - 3414937 - 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\Documents\Bot_sena_seguimiento\assets\Listados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C241FFCC-B929-4535-AD5A-E80B885346F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE51A8C2-4133-416D-8D25-9ECE7114E203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASISTENCIA " sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="365">
   <si>
     <r>
       <rPr>
@@ -1194,12 +1194,6 @@
     <t>Pereira Ávila</t>
   </si>
   <si>
-    <t xml:space="preserve">Sharith Yesid </t>
-  </si>
-  <si>
-    <t>González Rodríguez</t>
-  </si>
-  <si>
     <t>Danna Nicol</t>
   </si>
   <si>
@@ -1324,6 +1318,9 @@
   </si>
   <si>
     <t xml:space="preserve">Delicias de Amor </t>
+  </si>
+  <si>
+    <t>Budusitos</t>
   </si>
 </sst>
 </file>
@@ -2767,7 +2764,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="214">
+  <cellXfs count="215">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3295,6 +3292,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="51" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="16" borderId="67" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -42446,13 +42446,13 @@
         <v>32</v>
       </c>
       <c r="B9" s="58" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C9" s="58" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D9" s="58" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E9" s="58" t="s">
         <v>72</v>
@@ -42467,13 +42467,13 @@
         <v>75</v>
       </c>
       <c r="I9" s="58" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="J9" s="58" t="s">
         <v>76</v>
       </c>
       <c r="K9" s="58" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="L9" s="48"/>
       <c r="M9" s="48"/>
@@ -43211,7 +43211,7 @@
       </c>
       <c r="L24" s="48"/>
       <c r="M24" s="48" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="N24" s="48"/>
       <c r="O24" s="48"/>
@@ -43251,7 +43251,7 @@
       <c r="H25" s="84" t="s">
         <v>205</v>
       </c>
-      <c r="I25" s="82" t="s">
+      <c r="I25" s="214" t="s">
         <v>206</v>
       </c>
       <c r="J25" s="82">
@@ -43380,7 +43380,7 @@
         <v>19</v>
       </c>
       <c r="B28" s="81" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C28" s="95" t="s">
         <v>126</v>
@@ -43458,7 +43458,7 @@
       </c>
       <c r="L29" s="48"/>
       <c r="M29" s="48" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="N29" s="48"/>
       <c r="O29" s="48"/>
@@ -44097,7 +44097,7 @@
       </c>
       <c r="L42" s="48"/>
       <c r="M42" s="48" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="N42" s="48"/>
       <c r="O42" s="48"/>
@@ -44148,7 +44148,7 @@
       </c>
       <c r="L43" s="48"/>
       <c r="M43" s="48" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="N43" s="48"/>
       <c r="O43" s="48"/>
@@ -53011,11 +53011,12 @@
     <hyperlink ref="F39" r:id="rId71" xr:uid="{47CB2AD8-9FEB-42DA-94CA-F35FFA40E3FF}"/>
     <hyperlink ref="F22" r:id="rId72" xr:uid="{21AC6427-A11A-4A46-ACA5-32AE00815FCB}"/>
     <hyperlink ref="F40" r:id="rId73" xr:uid="{4F07F6D4-EEEA-444E-9ABD-73F7C92C1243}"/>
+    <hyperlink ref="I25" r:id="rId74" xr:uid="{FC0A317B-27AA-4EC1-8D42-4C7FE00C723E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId74"/>
+  <pageSetup orientation="landscape" r:id="rId75"/>
   <tableParts count="1">
-    <tablePart r:id="rId75"/>
+    <tablePart r:id="rId76"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -53072,7 +53073,7 @@
     </row>
     <row r="3" spans="1:6" ht="15.75">
       <c r="A3" s="210" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B3" s="66" t="s">
         <v>275</v>
@@ -53145,7 +53146,7 @@
     </row>
     <row r="10" spans="1:6" ht="15.75">
       <c r="A10" s="210" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B10" s="66" t="s">
         <v>284</v>
@@ -53172,26 +53173,20 @@
     <row r="12" spans="1:6" ht="15.75">
       <c r="A12" s="211"/>
       <c r="B12" s="66" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C12" s="66" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D12" s="113" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75">
       <c r="A13" s="211"/>
-      <c r="B13" s="66" t="s">
-        <v>291</v>
-      </c>
-      <c r="C13" s="66" t="s">
-        <v>292</v>
-      </c>
-      <c r="D13" s="113" t="s">
-        <v>158</v>
-      </c>
+      <c r="B13" s="66"/>
+      <c r="C13" s="66"/>
+      <c r="D13" s="113"/>
     </row>
     <row r="14" spans="1:6" ht="15.75">
       <c r="A14" s="212"/>
@@ -53215,7 +53210,7 @@
     </row>
     <row r="17" spans="1:4" ht="15.75">
       <c r="A17" s="210" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B17" s="66" t="s">
         <v>293</v>
@@ -53285,7 +53280,7 @@
     </row>
     <row r="24" spans="1:4" ht="15.75">
       <c r="A24" s="210" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B24" s="66" t="s">
         <v>302</v>
@@ -53315,7 +53310,7 @@
         <v>306</v>
       </c>
       <c r="C26" s="66" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D26" s="113" t="s">
         <v>131</v>
@@ -53355,7 +53350,7 @@
     </row>
     <row r="31" spans="1:4" ht="15.75">
       <c r="A31" s="210" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B31" s="66" t="s">
         <v>309</v>
@@ -53425,7 +53420,7 @@
     </row>
     <row r="38" spans="1:4" ht="15.75">
       <c r="A38" s="210" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B38" s="66" t="s">
         <v>317</v>
@@ -53443,7 +53438,7 @@
         <v>319</v>
       </c>
       <c r="C39" s="66" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D39" s="113" t="s">
         <v>143</v>
@@ -53464,13 +53459,13 @@
     <row r="41" spans="1:4" ht="15.75">
       <c r="A41" s="211"/>
       <c r="B41" s="66" t="s">
-        <v>322</v>
+        <v>288</v>
       </c>
       <c r="C41" s="66" t="s">
-        <v>323</v>
+        <v>289</v>
       </c>
       <c r="D41" s="113" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75">
@@ -53496,13 +53491,13 @@
     </row>
     <row r="45" spans="1:4" ht="15" customHeight="1">
       <c r="A45" s="210" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B45" s="66" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C45" s="66" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D45" s="113" t="s">
         <v>133</v>
@@ -53511,10 +53506,10 @@
     <row r="46" spans="1:4" ht="15" customHeight="1">
       <c r="A46" s="211"/>
       <c r="B46" s="66" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C46" s="66" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D46" s="113" t="s">
         <v>146</v>
@@ -53523,10 +53518,10 @@
     <row r="47" spans="1:4" ht="15" customHeight="1">
       <c r="A47" s="211"/>
       <c r="B47" s="66" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C47" s="66" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D47" s="113" t="s">
         <v>140</v>
@@ -53535,10 +53530,10 @@
     <row r="48" spans="1:4" ht="15" customHeight="1">
       <c r="A48" s="211"/>
       <c r="B48" s="66" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C48" s="66" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D48" s="113" t="s">
         <v>135</v>
@@ -53567,13 +53562,13 @@
     </row>
     <row r="52" spans="1:4" ht="15" customHeight="1">
       <c r="A52" s="210" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B52" s="66" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C52" s="66" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D52" s="113" t="s">
         <v>136</v>
@@ -53582,10 +53577,10 @@
     <row r="53" spans="1:4" ht="15" customHeight="1">
       <c r="A53" s="211"/>
       <c r="B53" s="66" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C53" s="66" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D53" s="113" t="s">
         <v>150</v>
@@ -53594,10 +53589,10 @@
     <row r="54" spans="1:4" ht="15" customHeight="1">
       <c r="A54" s="211"/>
       <c r="B54" s="66" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C54" s="66" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D54" s="113" t="s">
         <v>148</v>
@@ -53606,10 +53601,10 @@
     <row r="55" spans="1:4" ht="15" customHeight="1">
       <c r="A55" s="211"/>
       <c r="B55" s="66" t="s">
+        <v>336</v>
+      </c>
+      <c r="C55" s="66" t="s">
         <v>338</v>
-      </c>
-      <c r="C55" s="66" t="s">
-        <v>340</v>
       </c>
       <c r="D55" s="113" t="s">
         <v>144</v>
@@ -53618,10 +53613,10 @@
     <row r="56" spans="1:4" ht="15" customHeight="1" thickBot="1">
       <c r="A56" s="212"/>
       <c r="B56" s="68" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C56" s="68" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D56" s="118" t="s">
         <v>155</v>
@@ -53643,12 +53638,14 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="15" customHeight="1">
-      <c r="A59" s="210"/>
+      <c r="A59" s="210" t="s">
+        <v>364</v>
+      </c>
       <c r="B59" s="66" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C59" s="66" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D59" s="113" t="s">
         <v>138</v>
@@ -53657,10 +53654,10 @@
     <row r="60" spans="1:4" ht="15" customHeight="1">
       <c r="A60" s="211"/>
       <c r="B60" s="66" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C60" s="66" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D60" s="113" t="s">
         <v>156</v>
@@ -53704,35 +53701,34 @@
     <hyperlink ref="D6" r:id="rId4" xr:uid="{D14A4E92-C0E2-4696-BF8F-D8F4C20394FC}"/>
     <hyperlink ref="D10" r:id="rId5" xr:uid="{7598D655-2180-461C-9928-8BE1BFC7DC83}"/>
     <hyperlink ref="D11" r:id="rId6" xr:uid="{D5C00FFE-C863-4926-9205-AF8F08BEC239}"/>
-    <hyperlink ref="D12" r:id="rId7" xr:uid="{564CB0C5-9294-43C8-9F74-758633B923E8}"/>
-    <hyperlink ref="D13" r:id="rId8" xr:uid="{287BD786-4DED-4DBF-B6F3-AF9F422314C2}"/>
-    <hyperlink ref="D17" r:id="rId9" xr:uid="{E29BFCDD-27C7-4BBA-82F1-8DA1BB4BF5E0}"/>
-    <hyperlink ref="D18" r:id="rId10" xr:uid="{AF6534E7-3696-4873-84C8-6037A9BB6F8C}"/>
-    <hyperlink ref="D19" r:id="rId11" xr:uid="{335FE742-65B9-4738-B90A-0917A8AE3738}"/>
-    <hyperlink ref="D20" r:id="rId12" xr:uid="{D00ABF86-B5B6-4CF2-834B-208EB25AC884}"/>
-    <hyperlink ref="D24" r:id="rId13" xr:uid="{7EAB6215-249B-444D-9E1E-C71E6A387E5B}"/>
-    <hyperlink ref="D25" r:id="rId14" xr:uid="{1EEC0362-69F4-4457-9702-49517EF9B022}"/>
-    <hyperlink ref="D26" r:id="rId15" xr:uid="{836C440A-F077-4AE0-A519-1A7D133A6DA5}"/>
-    <hyperlink ref="D27" r:id="rId16" xr:uid="{62EB46EE-231C-4953-9AE3-D9DD2AD48658}"/>
-    <hyperlink ref="D31" r:id="rId17" xr:uid="{840E8B01-D584-4103-BCDC-1087897CD79F}"/>
-    <hyperlink ref="D32" r:id="rId18" xr:uid="{48F22200-13AE-4713-AE5B-423F84F70075}"/>
-    <hyperlink ref="D33" r:id="rId19" xr:uid="{1AC3C72B-2911-40D8-9DF1-A116DF0A84BC}"/>
-    <hyperlink ref="D34" r:id="rId20" xr:uid="{F0DAA9D4-4B78-4B96-A1F3-86171AEB6763}"/>
-    <hyperlink ref="D38" r:id="rId21" xr:uid="{525CC6A7-E041-40D7-890B-B8625400678D}"/>
-    <hyperlink ref="D39" r:id="rId22" xr:uid="{F2007303-9E1D-45D2-A959-97CE8081C45E}"/>
-    <hyperlink ref="D40" r:id="rId23" xr:uid="{634ED716-CF7B-45CA-939A-B631D3D6C0C0}"/>
-    <hyperlink ref="D41" r:id="rId24" xr:uid="{ACDFB16E-EFCD-4208-905F-72D0BE4233B4}"/>
-    <hyperlink ref="D45" r:id="rId25" xr:uid="{85A134AC-87E3-4A71-8F8B-2218D89B1CF7}"/>
-    <hyperlink ref="D46" r:id="rId26" xr:uid="{55BD9931-A487-4129-B613-D052B9D2E43A}"/>
-    <hyperlink ref="D47" r:id="rId27" xr:uid="{6E9F97FA-3140-4E41-A8BD-C7E8D3F86C7B}"/>
-    <hyperlink ref="D48" r:id="rId28" xr:uid="{0472DDC2-CBD4-4B04-8528-EA9BBA75F391}"/>
-    <hyperlink ref="D52" r:id="rId29" xr:uid="{10C1359B-FE2B-41CE-99BF-90A20059629F}"/>
-    <hyperlink ref="D53" r:id="rId30" xr:uid="{8AE6A0A2-716A-46F8-8441-68E9607A39C7}"/>
-    <hyperlink ref="D54" r:id="rId31" xr:uid="{D79013BE-C6A2-439D-9836-1E180BA23CBB}"/>
-    <hyperlink ref="D55" r:id="rId32" xr:uid="{75D666DD-10EC-4262-B05C-5B12DCA9EAC5}"/>
-    <hyperlink ref="D56" r:id="rId33" xr:uid="{EB07EF50-4E64-43BA-87CD-BB81127CCCB7}"/>
-    <hyperlink ref="D59" r:id="rId34" xr:uid="{80B3C828-94C9-4BC4-BFDA-AFE5E3F5B574}"/>
-    <hyperlink ref="D60" r:id="rId35" xr:uid="{BA2F860E-577E-42F3-A716-4F537F1889D0}"/>
+    <hyperlink ref="D17" r:id="rId7" xr:uid="{E29BFCDD-27C7-4BBA-82F1-8DA1BB4BF5E0}"/>
+    <hyperlink ref="D18" r:id="rId8" xr:uid="{AF6534E7-3696-4873-84C8-6037A9BB6F8C}"/>
+    <hyperlink ref="D19" r:id="rId9" xr:uid="{335FE742-65B9-4738-B90A-0917A8AE3738}"/>
+    <hyperlink ref="D20" r:id="rId10" xr:uid="{D00ABF86-B5B6-4CF2-834B-208EB25AC884}"/>
+    <hyperlink ref="D24" r:id="rId11" xr:uid="{7EAB6215-249B-444D-9E1E-C71E6A387E5B}"/>
+    <hyperlink ref="D25" r:id="rId12" xr:uid="{1EEC0362-69F4-4457-9702-49517EF9B022}"/>
+    <hyperlink ref="D26" r:id="rId13" xr:uid="{836C440A-F077-4AE0-A519-1A7D133A6DA5}"/>
+    <hyperlink ref="D27" r:id="rId14" xr:uid="{62EB46EE-231C-4953-9AE3-D9DD2AD48658}"/>
+    <hyperlink ref="D31" r:id="rId15" xr:uid="{840E8B01-D584-4103-BCDC-1087897CD79F}"/>
+    <hyperlink ref="D32" r:id="rId16" xr:uid="{48F22200-13AE-4713-AE5B-423F84F70075}"/>
+    <hyperlink ref="D33" r:id="rId17" xr:uid="{1AC3C72B-2911-40D8-9DF1-A116DF0A84BC}"/>
+    <hyperlink ref="D34" r:id="rId18" xr:uid="{F0DAA9D4-4B78-4B96-A1F3-86171AEB6763}"/>
+    <hyperlink ref="D38" r:id="rId19" xr:uid="{525CC6A7-E041-40D7-890B-B8625400678D}"/>
+    <hyperlink ref="D39" r:id="rId20" xr:uid="{F2007303-9E1D-45D2-A959-97CE8081C45E}"/>
+    <hyperlink ref="D40" r:id="rId21" xr:uid="{634ED716-CF7B-45CA-939A-B631D3D6C0C0}"/>
+    <hyperlink ref="D45" r:id="rId22" xr:uid="{85A134AC-87E3-4A71-8F8B-2218D89B1CF7}"/>
+    <hyperlink ref="D46" r:id="rId23" xr:uid="{55BD9931-A487-4129-B613-D052B9D2E43A}"/>
+    <hyperlink ref="D47" r:id="rId24" xr:uid="{6E9F97FA-3140-4E41-A8BD-C7E8D3F86C7B}"/>
+    <hyperlink ref="D48" r:id="rId25" xr:uid="{0472DDC2-CBD4-4B04-8528-EA9BBA75F391}"/>
+    <hyperlink ref="D52" r:id="rId26" xr:uid="{10C1359B-FE2B-41CE-99BF-90A20059629F}"/>
+    <hyperlink ref="D53" r:id="rId27" xr:uid="{8AE6A0A2-716A-46F8-8441-68E9607A39C7}"/>
+    <hyperlink ref="D54" r:id="rId28" xr:uid="{D79013BE-C6A2-439D-9836-1E180BA23CBB}"/>
+    <hyperlink ref="D55" r:id="rId29" xr:uid="{75D666DD-10EC-4262-B05C-5B12DCA9EAC5}"/>
+    <hyperlink ref="D56" r:id="rId30" xr:uid="{EB07EF50-4E64-43BA-87CD-BB81127CCCB7}"/>
+    <hyperlink ref="D59" r:id="rId31" xr:uid="{80B3C828-94C9-4BC4-BFDA-AFE5E3F5B574}"/>
+    <hyperlink ref="D60" r:id="rId32" xr:uid="{BA2F860E-577E-42F3-A716-4F537F1889D0}"/>
+    <hyperlink ref="D41" r:id="rId33" xr:uid="{2D726380-94CC-4CC1-AEB9-3D1F39E2F42D}"/>
+    <hyperlink ref="D12" r:id="rId34" xr:uid="{48A14C87-A122-4450-B388-7FDC011AEB35}"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>

</xml_diff>